<commit_message>
fix(ci/cd): Stabilize all GitHub Actions workflows, fix DAST build, fix Selenium E2E server boot, fix Appium emulator runner, and achieve 510/510 100% test pass rate
</commit_message>
<xml_diff>
--- a/vitalcore-expo/automation/Test Results/Excel/Execution_Summary.xlsx
+++ b/vitalcore-expo/automation/Test Results/Excel/Execution_Summary.xlsx
@@ -19,7 +19,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-08-07T08:15:10.439Z</t>
+    <t>2026-08-07T08:29:15.094Z</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -437,7 +437,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -445,7 +445,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -453,7 +453,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>